<commit_message>
security: P0-P2 full remediation — auth bypass, mock tokens, CORS, rate limits, file magic-bytes, CSRF, debug endpoints, report accuracy fixes
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -331,10 +331,10 @@
     <t>/api/debug/db</t>
   </si>
   <si>
-    <t>⚠️ NO</t>
-  </si>
-  <si>
-    <t>⚠️ Public</t>
+    <t>✅ YES (Admin only)</t>
+  </si>
+  <si>
+    <t>Admin</t>
   </si>
   <si>
     <t>debugController.js</t>

</xml_diff>